<commit_message>
feat: compact "Entry" export label and refine manual-pending metric
Export "Manual Entry Required" placeholder cells as the compact "Entry"
label (display-only; stored row values and in-app UI unchanged). Count
the manual-pending metric only across the client-facing Segment, RTPL
status, and Location columns. Refresh the pivot-template workbook.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/opencall-frontend/frontend/public/pivot-template.xlsx
+++ b/opencall-frontend/frontend/public/pivot-template.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\opencall\opencall-frontend\frontend\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194B9A13-2F58-4AE3-8EDF-01AF5DB98ADA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B279347A-BDCF-4EA3-B3B8-76F4075F8FC4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14205" activeTab="1" xr2:uid="{6FADA489-992B-47E7-930B-77F27B0696E2}"/>
   </bookViews>
   <sheets>
-    <sheet name="pivot" sheetId="2" r:id="rId1"/>
-    <sheet name="open plan" sheetId="1" r:id="rId2"/>
+    <sheet name="Pivot" sheetId="2" r:id="rId1"/>
+    <sheet name="Open Call" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'open plan'!$A$1:$Z$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Open Call'!$A$1:$Z$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId3"/>
+    <pivotCache cacheId="14" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -193,7 +193,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="DELL" refreshedDate="46189.486047800929" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="1" xr:uid="{5BDCAA74-1F0F-40E6-BCA6-0B19CED970D2}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:Z1048576" sheet="open plan"/>
+    <worksheetSource ref="A1:Z1048576" sheet="Open Call"/>
   </cacheSource>
   <cacheFields count="26">
     <cacheField name="S.no" numFmtId="0">
@@ -325,7 +325,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BD285A8E-EA28-475A-90FE-FC982077E17D}" name="PivotTable3" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BD285A8E-EA28-475A-90FE-FC982077E17D}" name="PivotTable3" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A4:C7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="26">
     <pivotField showAll="0"/>

</xml_diff>